<commit_message>
Corrige cobertura de orgaos estaduais Point C
</commit_message>
<xml_diff>
--- a/data/output/validacao_fontes_revalidado_visualmente.xlsx
+++ b/data/output/validacao_fontes_revalidado_visualmente.xlsx
@@ -540,13 +540,13 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:21</t>
+          <t>2026-05-28T09:07:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -592,13 +592,13 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:24</t>
+          <t>2026-05-28T09:07:20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -644,13 +644,13 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:29</t>
+          <t>2026-05-28T09:07:29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -696,13 +696,13 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:33</t>
+          <t>2026-05-28T09:07:33</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>480</v>
+        <v>435</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -756,13 +756,13 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:37</t>
+          <t>2026-05-28T09:07:40</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>782</v>
+        <v>741</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -794,7 +794,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.filadelfia.ba.gov.br/ver_noticias.php?note=1447</t>
+          <t>https://www.filadelfia.ba.gov.br/ver_noticias.php?note=1393</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -808,13 +808,13 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:42</t>
+          <t>2026-05-28T09:07:46</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>786</v>
+        <v>1525</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -823,12 +823,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Filadélfia</t>
+          <t>Paramirim</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Selo Ouro</t>
+          <t>JOÃO DE ALMEIDA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -846,7 +846,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.filadelfia.ba.gov.br/ver_noticias.php?note=1393</t>
+          <t>https://www.paramirim.ba.gov.br/texto/viceprefeito</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -860,13 +860,13 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:48</t>
+          <t>2026-05-28T09:07:49</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>848</v>
+        <v>1802</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -875,30 +875,38 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Guanambi</t>
+          <t>Santa Brígida</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Planejamento</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Composição da Coligação</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Elder Alves</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>seplange@santabrigida.ba.gov.br</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>(75) 99846-3135</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.guanambi.ba.gov.br/texto/viceprefeito</t>
+          <t>https://www.santabrigida.ba.gov.br/internas/prefeitura/?id=7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -907,18 +915,18 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:50</t>
+          <t>2026-05-28T09:08:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1038</v>
+        <v>1837</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -927,34 +935,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Itabela</t>
+          <t>Santa Rita de Cássia</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Maria Vânia Costa Santana Ferreira</t>
+          <t>Rita de Cássia</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>(73) 98117-3514</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.itabela.ba.gov.br/secretarias</t>
+          <t>https://santaritadecassia.ba.gov.br/prefeito</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -963,18 +967,18 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:54</t>
+          <t>2026-05-28T09:08:06</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1570</v>
+        <v>1915</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -983,30 +987,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Paramirim</t>
+          <t>Seabra</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>JOÃO DE ALMEIDA</t>
+          <t>Neto da Pousada</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>(75) 3331-1421</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.paramirim.ba.gov.br/texto/viceprefeito</t>
+          <t>https://seabra.ba.gov.br/o-prefeito?perfil=turista</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1015,18 +1023,18 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-28T04:54:57</t>
+          <t>2026-05-28T09:08:12</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1765</v>
+        <v>1968</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1035,12 +1043,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Riacho de Santana</t>
+          <t>Serra Preta</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1050,7 +1058,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>JOAO VITOR MARTINS LARANJEIRA</t>
+          <t>Mario Gonçalves Neto Av</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1058,7 +1066,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.riachodesantana.ba.gov.br/texto/o_prefeito</t>
+          <t>https://www.serrapreta.ba.gov.br/gabinete/2/vice-prefeito</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1072,27 +1080,27 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:00</t>
+          <t>2026-05-28T09:08:15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2393</v>
+        <v>2284</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Governo do Distrito Federal</t>
+          <t>Vera Cruz</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Desenvolvimento econômico</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1102,7 +1110,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Thales Mendes Ferreira</t>
+          <t>Adrian Araújo Pereira Silva</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1110,7 +1118,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.df.gov.br/secretarias/</t>
+          <t>https://veracruz.ba.gov.br/sefaz-secretaria-da-fazenda?perfil=servidor</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1124,13 +1132,13 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:10</t>
+          <t>2026-05-28T09:08:19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2430</v>
+        <v>2366</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1184,13 +1192,13 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:13</t>
+          <t>2026-05-28T09:08:23</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2574</v>
+        <v>2561</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1204,7 +1212,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1214,7 +1222,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SA Superintendência</t>
+          <t>Gilson Daniel Batista</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1222,7 +1230,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://guacui.es.gov.br/chefia-de-gabinete.html</t>
+          <t>https://guacui.es.gov.br/superintendencia-de-financas/orgao-vinculado.html</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1236,13 +1244,13 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:25</t>
+          <t>2026-05-28T09:08:34</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2640</v>
+        <v>2781</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1251,12 +1259,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Guaçuí</t>
+          <t>Rio Bananal</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1266,7 +1274,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Guaçuí Vera Costa</t>
+          <t>LEGISLATURA PERÍODO</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1274,7 +1282,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://guacui.es.gov.br/superintendencia-de-financas/organograma.html</t>
+          <t>https://riobananal.es.gov.br/prefeitos</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1288,13 +1296,13 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:36</t>
+          <t>2026-05-28T09:08:38</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2642</v>
+        <v>2865</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1303,30 +1311,38 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Guaçuí</t>
+          <t>Venda Nova do Imigrante</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Vera Costa</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Tânia Aparecida Uliana Torres</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>gabinete@vendanova.es.gov.br</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>(28) 99905-7214; (28) 99937-6770</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://guacui.es.gov.br/superintendencia-de-financas/organograma.html</t>
+          <t>https://www.vendanova.es.gov.br/prefeito.php</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1335,18 +1351,18 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:36</t>
+          <t>2026-05-28T09:08:41</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2684</v>
+        <v>2880</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1355,30 +1371,30 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Guaçuí</t>
+          <t>Viana</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>planejamento@guacui.es.gov.br</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Rafael Oliveira Kirmse</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://guacui.es.gov.br/secretaria-de-planejamento/orgao-vinculado.html</t>
+          <t>https://viana.es.gov.br/secretaria</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1392,27 +1408,27 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:47</t>
+          <t>2026-05-28T09:08:45</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2698</v>
+        <v>2904</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ibatiba</t>
+          <t>Abadia de Goiás</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1420,17 +1436,17 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>fazendaibatiba@gmail.com</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Wander Saraiva de Carvalho</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.ibatiba.es.gov.br/secretaria/ler/17/-secretaria-municipal-de-fazenda</t>
+          <t>https://abadiadegoias.go.gov.br/estrutura/gabinete-do-prefeito/</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1444,45 +1460,53 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:49</t>
+          <t>2026-05-28T09:08:53</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2930</v>
+        <v>2910</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Vargem Alta</t>
+          <t>Abadia de Goiás</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Desenvolvimento econômico</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>EMERSON CEREZA SOUZA</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>Maria do Carmo de Queiroz Souza</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>gabinete@abadiadegoias.go.gov.br</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>(62) 99348-0641</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.vargemalta.es.gov.br/secretaria</t>
+          <t>https://abadiadegoias.go.gov.br/estrutura/gabinete-do-prefeito/</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1491,18 +1515,18 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:52</t>
+          <t>2026-05-28T09:08:53</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2979</v>
+        <v>3201</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1511,7 +1535,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Abadia de Goiás</t>
+          <t>Itaberaí</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1521,20 +1545,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wander Saraiva de Carvalho</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
+          <t>Rita de Cássia Soares Mendonça</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>gabinete@itaberai.go.gov.br</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://abadiadegoias.go.gov.br/estrutura/gabinete-do-prefeito/</t>
+          <t>https://itaberai.go.gov.br/gabinete-da-prefeita/</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1543,18 +1571,18 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:57</t>
+          <t>2026-05-28T09:08:57</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2982</v>
+        <v>3515</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1563,12 +1591,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Abadia de Goiás</t>
+          <t>Silvânia</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1578,7 +1606,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ortopedia Brasil</t>
+          <t>Fábio André da Silva</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1586,7 +1614,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://abadiadegoias.go.gov.br/estrutura/gabinete-do-prefeito/</t>
+          <t>https://silvania.go.gov.br/estrutura/gabinete-do-vice-prefeito-2/</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1600,13 +1628,13 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-05-28T04:55:57</t>
+          <t>2026-05-28T09:09:03</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3220</v>
+        <v>3529</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1615,12 +1643,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Goiânia</t>
+          <t>São João d'Aliança</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1630,7 +1658,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sandro Mabel</t>
+          <t>Shirley Araújo da Paz</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1638,7 +1666,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.goiania.go.gov.br/sing_prefeitura/prefeito/</t>
+          <t>https://www.saojoaodalianca.go.gov.br/estrutura/gabinete-da-prefeita/chefia-de-gabinete/</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1652,13 +1680,13 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:00</t>
+          <t>2026-05-28T09:09:11</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3303</v>
+        <v>3559</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1667,22 +1695,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Itaberaí</t>
+          <t>São Simão</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Thayane Silva Rodrigues Moreira</t>
+          <t>Janaina Camila da Costa</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1690,7 +1718,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://itaberai.go.gov.br/gabinete-vice-prefeito/</t>
+          <t>https://saosimao.go.gov.br/estrutura/secretaria-de-administracao/chefia-de-gabinete-10/</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1704,45 +1732,49 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:04</t>
+          <t>2026-05-28T09:09:17</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3572</v>
+        <v>3661</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Santa Helena de Goiás</t>
+          <t>Alpinópolis</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Chefe de gabinete</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Dinair Maria Rosa Vieira</t>
+          <t>Rafael Henrique da Silva Freire</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>(35) 3523-1808</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.santahelena.go.gov.br/estrutura-organizacional/?id=1</t>
+          <t>https://alpinopolis.mg.gov.br/prefeito/</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1751,27 +1783,27 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:09</t>
+          <t>2026-05-28T09:09:20</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3597</v>
+        <v>4409</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Silvânia</t>
+          <t>Ibiá</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1786,7 +1818,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Carlos José Mayer dos Santos</t>
+          <t>Lívia Maria Pimenta Rodrigues Reis</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1794,7 +1826,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://silvania.go.gov.br/estrutura/gabinete-do-prefeito-2/</t>
+          <t>https://www.ibia.mg.gov.br/secretaria-municipal-de-gabinete-do-prefeito/</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -1808,13 +1840,13 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:13</t>
+          <t>2026-05-28T09:09:27</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3754</v>
+        <v>5102</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1823,34 +1855,30 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Alpinópolis</t>
+          <t>Ouro Preto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Rafael Henrique da Silva Freire</t>
+          <t>Camila Sardinha Cecconello</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>(35) 3523-1808</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://alpinopolis.mg.gov.br/prefeito/</t>
+          <t>https://www.ouropreto.mg.gov.br/desenvolvimentourbano/conheca-secretaria</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -1859,18 +1887,18 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:16</t>
+          <t>2026-05-28T09:09:30</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3823</v>
+        <v>5820</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1879,7 +1907,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Araçuaí</t>
+          <t>Turmalina</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1894,7 +1922,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>KELVIO MARCILIO SILVA OLIVEIRA</t>
+          <t>Warlen Francisco Da Silva</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -1902,7 +1930,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.aracuai.mg.gov.br/prefeitura/vice-prefeito</t>
+          <t>https://www.turmalina.mg.gov.br/vices</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -1916,22 +1944,22 @@
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:24</t>
+          <t>2026-05-28T09:09:34</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3872</v>
+        <v>5958</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Barbacena</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1946,7 +1974,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Carlos Augusto Soares</t>
+          <t>ABILIO JACQUES BRUNINI MOUMER</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1954,7 +1982,7 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www1.barbacena.mg.gov.br/portal/prefeito/13/1</t>
+          <t>https://cuiaba.mt.gov.br/a-prefeitura/o-prefeito</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -1968,49 +1996,45 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:26</t>
+          <t>2026-05-28T09:09:37</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4006</v>
+        <v>6026</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Brumadinho</t>
+          <t>Altônia</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Desenvolvimento econômico</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Andre Luiz Giovannini Paiva</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>prefeito@altonia.pr.gov.br</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>(31) 97222-6355</t>
-        </is>
-      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://novo.brumadinho.mg.gov.br/portal/departamento/secretaria-de-desenvolvimento-economico</t>
+          <t>https://www.altonia.pr.gov.br/secretariaView/1_Prefeito-Municipal.html</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2019,50 +2043,54 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:31</t>
+          <t>2026-05-28T09:09:42</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4127</v>
+        <v>6163</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Carangola</t>
+          <t>Bituruna</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Natural de Carangola</t>
+          <t>Eneias Santos Mello</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>(42) 3553-8602</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.carangola.mg.gov.br/prefeitura/prefeito-vice-prefeito</t>
+          <t>https://www.bituruna.pr.gov.br/secretariaView/?id=40</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2071,32 +2099,32 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:39</t>
+          <t>2026-05-28T09:09:46</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4359</v>
+        <v>6468</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Divino</t>
+          <t>Faxinal</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2106,7 +2134,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CARLOS ROBERTO ROCHA</t>
+          <t>Ismael Pinto Siqueira</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -2114,7 +2142,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.divino.mg.gov.br/prefeitura/vice-prefeito</t>
+          <t>https://www.faxinal.pr.gov.br/presidentes</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2128,49 +2156,45 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:46</t>
+          <t>2026-05-28T09:09:52</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4609</v>
+        <v>6593</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Itamarandiba</t>
+          <t>Ibiporã</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Planejamento</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Flaviana Edneia Leandro</t>
+          <t>LUCIANA MASSON</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>7602-2633</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.itamarandiba.mg.gov.br/scretarias/114-secretaria-municipal-de-financas.html?tmpl=component&amp;print=1&amp;layout=default</t>
+          <t>https://www.ibipora.pr.gov.br/secretariaView/?id=18</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2179,32 +2203,32 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:52</t>
+          <t>2026-05-28T09:09:56</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>6069</v>
+        <v>6597</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Ibiporã</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Planejamento</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2214,7 +2238,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>ABILIO JACQUES BRUNINI MOUMER</t>
+          <t>JUAREZ AFONSO IGNÁCIO</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -2222,7 +2246,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://cuiaba.mt.gov.br/a-prefeitura/o-prefeito</t>
+          <t>https://www.ibipora.pr.gov.br/secretariaView/?id=13</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2236,13 +2260,13 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:55</t>
+          <t>2026-05-28T09:10:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>6186</v>
+        <v>6770</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2251,12 +2275,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Altônia</t>
+          <t>Mandaguaçu</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2264,17 +2288,17 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>prefeito@altonia.pr.gov.br</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Federais e Estaduais</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.altonia.pr.gov.br/secretariaView/1_Prefeito-Municipal.html</t>
+          <t>https://www.mandaguacu.pr.gov.br/prefeitura/detalhe-departamento/50/chefe-de-gabinete/</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2288,13 +2312,13 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-05-28T04:56:59</t>
+          <t>2026-05-28T09:10:05</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>6260</v>
+        <v>6833</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2303,12 +2327,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Arapoti</t>
+          <t>Maringá</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2318,7 +2342,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>TALITA TEIXEIRA KLUPPEL DOS SANTOS</t>
+          <t>Sandra Jacovós</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -2326,7 +2350,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.arapoti.pr.gov.br/prefeitura/detalhe-departamento/53/planejamento/</t>
+          <t>https://www.maringa.pr.gov.br/prefeitos/silvio-barros/42</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2340,13 +2364,13 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:04</t>
+          <t>2026-05-28T09:10:10</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>6348</v>
+        <v>7247</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2355,34 +2379,30 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cafelândia</t>
+          <t>Sengés</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Diziely Rocha de Ré</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>planejamento@cafelandia.pr.gov.br</t>
-        </is>
-      </c>
+          <t>CARLOS EDUARDO FUZETO</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.cafelandia.pr.gov.br//index.php?sessao=b054603368xwb0&amp;id=3942</t>
+          <t>https://www.senges.pr.gov.br/portal/secretariasP.php</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2391,32 +2411,32 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:07</t>
+          <t>2026-05-28T09:10:14</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>6406</v>
+        <v>7415</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Campo Magro</t>
+          <t>Araruama</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2426,7 +2446,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Geovana Boza Kmiecik</t>
+          <t>Daniela Cuinse Abreu Soares</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2434,7 +2454,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.campomagro.pr.gov.br/secretariasAll</t>
+          <t>https://www.araruama.rj.gov.br/public/a-prefeitura/prefeita</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2448,27 +2468,27 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:11</t>
+          <t>2026-05-28T09:10:21</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>6537</v>
+        <v>8132</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Contenda</t>
+          <t>Natal</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Agências municipais de desenvolvimento</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2476,25 +2496,17 @@
           <t>Encontrado</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Márcia Maria Cionek de Carvalho</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>financeiro@contenda.pr.gov.br</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>(41) 3625-1212</t>
-        </is>
-      </c>
+          <t>saladoempreendedor@natal.rn.gov.br</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.contenda.pr.gov.br/secretarias/</t>
+          <t>https://saladoempreendedor.natal.rn.gov.br/inicio.php</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2503,32 +2515,32 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:16</t>
+          <t>2026-05-28T09:10:24</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>6741</v>
+        <v>8134</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ibiporã</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2538,7 +2550,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Paulo Balconi</t>
+          <t>Leonardo Barreto de Moraes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -2546,7 +2558,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.ibipora.pr.gov.br/secretariaView/?id=25</t>
+          <t>https://transparencia.portovelho.ro.gov.br/despesas/despesas/149693ea-d294-4a75-ac9a-0b2700eaf822</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2560,22 +2572,22 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:19</t>
+          <t>2026-05-28T09:10:27</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>6742</v>
+        <v>8157</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ibiporã</t>
+          <t>Agudo</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2585,20 +2597,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>JUNIOR FREDERICO ALIANO</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>Encontrado</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>fazenda@agudo.rs.gov.br; contabilidade@agudo.rs.gov.br</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.ibipora.pr.gov.br/secretariaView/?id=23</t>
+          <t>https://www.agudo.rs.gov.br/secretarias/sec-da-fazenda-1</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2607,50 +2619,58 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:22</t>
+          <t>2026-05-28T09:10:36</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>6748</v>
+        <v>8558</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ibiporã</t>
+          <t>Gramado</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>LEILIANE DE JESUS</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+          <t>Luia Barbacovi</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>gabinete@gramado.rs.gov.br</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>(54) 3286-0200</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.ibipora.pr.gov.br/secretariaView/?id=16</t>
+          <t>https://gramado.atende.net/subportal/gabinete-do-prefeito</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2659,32 +2679,32 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:26</t>
+          <t>2026-05-28T09:10:40</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>6753</v>
+        <v>8938</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ibiporã</t>
+          <t>Sananduva</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2694,7 +2714,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GUSTAVO TONELI DE SÁ</t>
+          <t>Tiago Tomielo</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2702,7 +2722,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.ibipora.pr.gov.br/secretariaView/?id=6</t>
+          <t>https://www.sananduva.rs.gov.br/pg.php?area=GABINETEDOPREFEITO</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -2716,27 +2736,27 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:29</t>
+          <t>2026-05-28T09:10:44</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>6940</v>
+        <v>8968</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mandaguaçu</t>
+          <t>Santa Maria</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Chefe de gabinete</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2746,7 +2766,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Adauto Almir Braz</t>
+          <t>Rodrigo Decimo</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2754,7 +2774,7 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://www.mandaguacu.pr.gov.br/prefeitura/departamento</t>
+          <t>https://www.santamaria.rs.gov.br/sepe</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -2768,53 +2788,45 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:33</t>
+          <t>2026-05-28T09:10:51</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>7076</v>
+        <v>8976</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Morretes</t>
+          <t>Santa Maria</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sueli Pilar</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>gabinete@morretes.pr.gov.br</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>(41) 3462-1266</t>
-        </is>
-      </c>
+          <t>Sub Menus</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.morretes.pr.gov.br/secretariaView/15_gabinete-institucional.html</t>
+          <t>https://www.santamaria.rs.gov.br/smdei/1203-desenvolvimento-econ%C3%B4mico</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -2823,54 +2835,50 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:38</t>
+          <t>2026-05-28T09:10:56</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>7130</v>
+        <v>9072</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Paiçandu</t>
+          <t>Sarandi</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Natalia Caroline Pereira Casarotto</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>planejamento@paicandu.pr.gov.br</t>
-        </is>
-      </c>
+          <t>Amauri Braga</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>https://paicandu.pr.gov.br/index.php?sessao=b054603368xwb0&amp;id=3507</t>
+          <t>https://sarandi.rs.gov.br/institucional/vice-prefeito/</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -2879,50 +2887,54 @@
         </is>
       </c>
       <c r="L46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:41</t>
+          <t>2026-05-28T09:11:01</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>7296</v>
+        <v>9301</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Quitandinha</t>
+          <t>Teutônia</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Desenvolvimento</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Antonio Iargas</t>
+          <t>Renato Airton Altmann</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>(51) 3762-7700</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.quitandinha.pr.gov.br/administracao</t>
+          <t>https://teutonia.rs.gov.br/</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -2931,88 +2943,88 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:44</t>
+          <t>2026-05-28T09:11:10</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>7455</v>
+        <v>9452</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>São Mateus do Sul</t>
+          <t>Abelardo Luz</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Desenvolvimento econômico</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Carlos Roberto Chaves</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>industriaecomercio@saomateusdosul.pr.gov.br</t>
-        </is>
-      </c>
+          <t>Antonio Nadin</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://www.saomateusdosul.pr.gov.br/portal/secretarias/29/desenvolvimento-economico</t>
+          <t>https://abelardoluz.sc.gov.br/pagina-7345/</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Não validado</t>
         </is>
       </c>
       <c r="L48" t="n">
-        <v>2</v>
-      </c>
-      <c r="M48" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Fonte não validável no momento: Bloqueio técnico. HTTP 403. | HTTP 403.</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:47</t>
+          <t>2026-05-28T09:11:17</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>7584</v>
+        <v>9980</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Araruama</t>
+          <t>Lages</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3022,7 +3034,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Daniela Cuinse Abreu Soares</t>
+          <t>Jair da Costa Teixeira Junior</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -3030,7 +3042,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.araruama.rj.gov.br/public/a-prefeitura/prefeita</t>
+          <t>https://www.lages.sc.gov.br/vice-prefeito</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3044,22 +3056,22 @@
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:51</t>
+          <t>2026-05-28T09:11:23</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>7844</v>
+        <v>10287</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Magé</t>
+          <t>São Miguel do Oeste</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3072,25 +3084,17 @@
           <t>Encontrado</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>GUSTAVO DA COSTA COZZOLINO</t>
-        </is>
-      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>desenvolvimento@mage.rj.gov.br</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>(21) 2317-0208</t>
-        </is>
-      </c>
+          <t>economico2@saomiguel.sc.gov.br</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://mage.rj.gov.br/departamentos-e-secretarias/</t>
+          <t>https://www.saomiguel.sc.gov.br/paginas/desenvolvimento-economico</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3099,32 +3103,32 @@
         </is>
       </c>
       <c r="L50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-05-28T04:57:55</t>
+          <t>2026-05-28T09:11:32</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>7908</v>
+        <v>10387</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Natividade</t>
+          <t>Aracaju</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3134,7 +3138,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Marcos Antônio</t>
+          <t>Emília Corrêa</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
@@ -3142,7 +3146,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://www.natividade.rj.gov.br/prefeitura/prefeito</t>
+          <t>https://www.aracaju.se.gov.br/viceprefeito/</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3156,27 +3160,27 @@
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:03</t>
+          <t>2026-05-28T09:11:34</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>7910</v>
+        <v>10392</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Natividade</t>
+          <t>Aracaju</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3186,7 +3190,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Cláudio Leite</t>
+          <t>Mayara Pinto Teixeira</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -3194,7 +3198,7 @@
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
-          <t>https://www.natividade.rj.gov.br/prefeitura/vice-prefeito</t>
+          <t>https://www.aracaju.se.gov.br/fazenda/estrutura_administrativa/</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3208,45 +3212,45 @@
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:10</t>
+          <t>2026-05-28T09:11:37</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>8310</v>
+        <v>10492</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Natal</t>
+          <t>Itabaiana</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Agências municipais de desenvolvimento</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>saladoempreendedor@natal.rn.gov.br</t>
+          <t>gabinete@itabaiana.se.gov.br</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>https://saladoempreendedor.natal.rn.gov.br/inicio.php</t>
+          <t>https://itabaiana.se.gov.br/departamento/gabinete-do-prefeito?export_data=json</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3260,45 +3264,53 @@
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:13</t>
+          <t>2026-05-28T09:11:41</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>8322</v>
+        <v>10494</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Porto Velho</t>
+          <t>Itabaiana</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Leonardo Barreto de Moraes</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+          <t>Maria de Lourdes Machado Bispo</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>gabinete@itabaiana.se.gov.br</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>(79) 3431-9701</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
-          <t>https://transparencia.portovelho.ro.gov.br/despesas/despesas/149693ea-d294-4a75-ac9a-0b2700eaf822</t>
+          <t>https://itabaiana.se.gov.br/departamento/20/chefe-de-gabinete?export_data=xml</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3307,50 +3319,50 @@
         </is>
       </c>
       <c r="L54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:16</t>
+          <t>2026-05-28T09:11:44</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>8363</v>
+        <v>10702</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Agudo</t>
+          <t>Adamantina</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>fazenda@agudo.rs.gov.br; contabilidade@agudo.rs.gov.br</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>José Carlos Martins Tiveron</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://www.agudo.rs.gov.br/secretarias/sec-da-fazenda-1</t>
+          <t>https://www.adamantina.sp.gov.br/portal/prefeito/13/1</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3359,54 +3371,50 @@
         </is>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:23</t>
+          <t>2026-05-28T09:11:48</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>8578</v>
+        <v>10876</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Caçapava do Sul</t>
+          <t>Bariri</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Marcelo Spode</t>
+          <t>Paulo Kezo</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>(55) 3398-0040</t>
-        </is>
-      </c>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
-          <t>https://www.cacapavadosul.rs.gov.br/administracao&amp;secretaria=prefeito</t>
+          <t>https://www.bariri.sp.gov.br/portal/prefeito/14/2</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3415,54 +3423,50 @@
         </is>
       </c>
       <c r="L56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:28</t>
+          <t>2026-05-28T09:11:51</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>8725</v>
+        <v>10904</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Flores da Cunha</t>
+          <t>Barrinha</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Desenvolvimento econômico</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Vivian Schiavenin</t>
+          <t>Ludovico José Homem Marcari</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>(54) 99266-4656</t>
-        </is>
-      </c>
+      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://www.floresdacunha.rs.gov.br/secao_administracao.php?id=53</t>
+          <t>https://portal.barrinha.sp.gov.br/prefeito/</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -3471,32 +3475,32 @@
         </is>
       </c>
       <c r="L57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:33</t>
+          <t>2026-05-28T09:12:19</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>8891</v>
+        <v>11342</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Jaguarão</t>
+          <t>Guararapes</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Vice-prefeito</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3506,7 +3510,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Diego Coronel Gonzalez</t>
+          <t>Eduardo Zanetti</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
@@ -3514,7 +3518,7 @@
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://www.jaguarao.rs.gov.br/secretarias/secretaria-da-fazenda/</t>
+          <t>https://www.guararapes.sp.gov.br/portal/prefeito/13/2</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -3528,22 +3532,22 @@
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:36</t>
+          <t>2026-05-28T09:12:22</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>8985</v>
+        <v>11401</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Novo Hamburgo</t>
+          <t>Guaíra</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3553,24 +3557,20 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Encontrado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Daiana de Leonço Monzon</t>
+          <t>Josias Domingos Silva</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>(51) 3097-9400</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://www.novohamburgo.rs.gov.br/smdei</t>
+          <t>https://www.guaira.sp.gov.br/prefeitura/detalhe-departamento/40/desenvolvimento-economico/</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -3579,32 +3579,32 @@
         </is>
       </c>
       <c r="L59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:39</t>
+          <t>2026-05-28T09:12:26</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>9233</v>
+        <v>11466</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Santo Antônio da Patrulha</t>
+          <t>Indaiatuba</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3612,17 +3612,17 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>gabinete@santoantoniodapatrulha.rs.gov.br</t>
-        </is>
-      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Instalação e Ampliação</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
-          <t>https://www.santoantoniodapatrulha.rs.gov.br/prefeito-e-vice/prefeito/</t>
+          <t>https://www.indaiatuba.sp.gov.br/desenvolvimento-economico-industria-comercio-e-turismo/incentivos-fiscais/tramitacao/</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -3636,27 +3636,27 @@
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:47</t>
+          <t>2026-05-28T09:12:28</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>9380</v>
+        <v>11743</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>São Jerônimo</t>
+          <t>Leme</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Filipe Almeida Pico</t>
+          <t>CARLOS ANTONIO DINIZ</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -3674,7 +3674,7 @@
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.saojeronimo.rs.gov.br/gabinete-do-prefeito//?gabinete-do-prefeito.html</t>
+          <t>https://www.leme.sp.gov.br/prefeitura/gabinete</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -3688,27 +3688,27 @@
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:54</t>
+          <t>2026-05-28T09:12:31</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>9393</v>
+        <v>11746</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>São Jerônimo</t>
+          <t>Leme</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3718,23 +3718,19 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Diogo Lima</t>
+          <t>Vera Regina Pilon Rodrigues Penteado</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>planejamento@saojeronimo.rs.gov.br</t>
+          <t>financas@leme.sp.gov.br</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>(51) 99576-5288</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
-          <t>https://www.saojeronimo.rs.gov.br/setor/visualizar/id/1021/?coordenadoria-de-planejamento.html</t>
+          <t>https://www.leme.sp.gov.br/secretarias/secretaria-de-financas-3</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -3743,27 +3739,27 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:57</t>
+          <t>2026-05-28T09:12:33</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>9484</v>
+        <v>11791</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Tapejara</t>
+          <t>Louveira</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3778,7 +3774,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Vilmar Merotto</t>
+          <t>Posto de Sa</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
@@ -3786,7 +3782,7 @@
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://tapejara.rs.gov.br/municipio/prefeitos</t>
+          <t>https://www.louveira.sp.gov.br/prefeitos</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -3800,83 +3796,83 @@
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr">
         <is>
-          <t>2026-05-28T04:58:59</t>
+          <t>2026-05-28T09:12:37</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>9667</v>
+        <v>11975</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Abelardo Luz</t>
+          <t>Osasco</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Planejamento</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Antonio Nadin</t>
+          <t>Juliano Duarte Vieira</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>(11) 3652-9505; 2182-1137</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
-          <t>https://abelardoluz.sc.gov.br/pagina-7345/</t>
+          <t>https://osasco.sp.gov.br/secretarias/</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Não validado</t>
+          <t>Validado</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>Fonte não validável no momento: Bloqueio técnico. HTTP 403. | HTTP 403.</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:02</t>
+          <t>2026-05-28T09:12:41</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>9890</v>
+        <v>12068</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Chapecó</t>
+          <t>Pindamonhangaba</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3884,17 +3880,17 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>fazenda@chapeco.sc.gov.br</t>
-        </is>
-      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Rodrigo Lóssio Ferreira</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://www.chapeco.sc.gov.br/conteudo/23/secretaria-de-fazenda</t>
+          <t>https://www.pindamonhangaba.sp.gov.br/gabinete</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -3908,109 +3904,97 @@
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:05</t>
+          <t>2026-05-28T09:12:44</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>9921</v>
+        <v>12302</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Correia Pinto</t>
+          <t>Rio das Pedras</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Jaison Muniz Rosa</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>financas@correiapinto.sc.gov.br</t>
+          <t>prefeito@riodaspedras.sp.gov.br</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
-          <t>https://correiapinto.sc.gov.br/estrutura-organizacional/</t>
+          <t>https://www.riodaspedras.sp.gov.br/prefeito.php?FiltroSecretaria=8</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Não validado</t>
+          <t>Validado</t>
         </is>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>Fonte não validável no momento: Bloqueio técnico. HTTP 403. | HTTP 403.</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:07</t>
+          <t>2026-05-28T09:12:57</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>10098</v>
+        <v>12303</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Itajaí</t>
+          <t>Rio das Pedras</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Chefe de gabinete</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>André Sandri</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>(47) 3341-6024</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>prefeito@riodaspedras.sp.gov.br</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://www.itajai.sc.gov.br/e/94</t>
+          <t>https://www.riodaspedras.sp.gov.br/prefeitos.php</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4019,32 +4003,32 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:10</t>
+          <t>2026-05-28T09:13:03</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>10611</v>
+        <v>12504</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Aracaju</t>
+          <t>Suzano</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Prefeito</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -4054,7 +4038,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Emília Corrêa</t>
+          <t>Criminal de Ferraz</t>
         </is>
       </c>
       <c r="G68" t="inlineStr"/>
@@ -4062,7 +4046,7 @@
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://www.aracaju.se.gov.br/viceprefeito/</t>
+          <t>https://suzano.sp.gov.br/gabinete-do-prefeito/afranio-evaristo-da-silva/</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4076,27 +4060,27 @@
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:13</t>
+          <t>2026-05-28T09:13:06</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>10904</v>
+        <v>12627</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>São Cristóvão</t>
+          <t>São Miguel Arcanjo</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4106,7 +4090,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Carlyane dos Santos</t>
+          <t>RODOLFO KENJI ESPIRITO SANTO</t>
         </is>
       </c>
       <c r="G69" t="inlineStr"/>
@@ -4114,7 +4098,7 @@
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.saocristovao.se.gov.br/orgaos/gapre</t>
+          <t>https://www.saomiguelarcanjo.sp.gov.br/prefeitura/departamento</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4128,13 +4112,13 @@
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:16</t>
+          <t>2026-05-28T09:13:12</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>10935</v>
+        <v>12773</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -4143,7 +4127,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Adamantina</t>
+          <t>Valinhos</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4156,17 +4140,17 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>José Carlos Martins Tiveron</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>gabinetedoprefeito@valinhos.sp.gov.br</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://www.adamantina.sp.gov.br/portal/prefeito/13/1</t>
+          <t>https://www.valinhos.sp.gov.br/portal/prefeito/13/1</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4180,13 +4164,13 @@
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:19</t>
+          <t>2026-05-28T09:13:15</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>10956</v>
+        <v>12812</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -4195,30 +4179,30 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Agudos</t>
+          <t>Vinhedo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Romildo Virgilino dos Santos</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr"/>
+          <t>Encontrado</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>patemprego@vinhedo.sp.gov.br</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://www.agudos.sp.gov.br/prefeitura/detalhe-departamento/28/gabinete-do-prefeito/</t>
+          <t>https://www.vinhedo.sp.gov.br/portal/secretarias/25/desenvolvimento-economico/portal/internautas/cadastrar/chamados</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4232,97 +4216,105 @@
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:24</t>
+          <t>2026-05-28T09:13:19</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>11243</v>
+        <v>12911</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Botucatu</t>
+          <t>Secretaria de Desenvolvimento Economico, Trabalho e Renda do Distrito Federal</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Fábio Vieira</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+          <t>Encontrado</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>ilton.teixeira@sedet.df.gov.br; alex.souza@sedet.df.gov.br; hilda.silva@sedet.df.gov.br; danielle.alves@sedet.df.gov.br; veronica.lisboa@sedet.df.gov.br</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>(61) 3773-9338; (61) 3773-9478; (61) 3773-9313; (61) 3773-9357; (61) 3773-9528</t>
+        </is>
+      </c>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
-          <t>https://www.botucatu.sp.gov.br/prefeitura</t>
+          <t>https://www.sedet.df.gov.br/subsecretarias?p_p_id=com_liferay_login_web_portlet_LoginPortlet&amp;p_p_lifecycle=1&amp;p_p_state=normal&amp;p_p_state_rcv=1&amp;p_auth=kez8ZWJE</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Validado</t>
+          <t>Não validado</t>
         </is>
       </c>
       <c r="L72" t="n">
-        <v>1</v>
-      </c>
-      <c r="M72" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>Fonte não validável no momento: Bloqueio técnico. HTTP 403. | HTTP 403.</t>
+        </is>
+      </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:28</t>
+          <t>2026-05-28T09:13:22</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>11762</v>
+        <v>12952</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Itapetininga</t>
+          <t>Secretaria de Estado de Industria e Comercio do Maranhao</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Chefe de gabinete</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>secretariafinancas@itapetininga.sp.gov.br; financas@itapetininga.sp.gov.br; itapecontabil@itapetininga.sp.gov.br</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Kaud Abdalla</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.itapetininga.sp.gov.br/prefeitura/detalhe-departamento/10/financas/</t>
+          <t>https://seinc.ma.gov.br/quem-e-quem</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -4331,54 +4323,50 @@
         </is>
       </c>
       <c r="L73" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:31</t>
+          <t>2026-05-28T09:14:04</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>11988</v>
+        <v>13011</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Leme</t>
+          <t>Secretaria de Meio Ambiente, Desenvolvimento, Ciencia, Tecnologia e Inovacao de Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Finanças/Fazenda</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>Vera Regina Pilon Rodrigues Penteado</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>financas@leme.sp.gov.br</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr"/>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>(67) 3318-5057</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
-          <t>https://www.leme.sp.gov.br/secretarias/secretaria-de-financas-3</t>
+          <t>https://www.semadesc.ms.gov.br/unidade-administrativa/superintendencia-de-administracao/</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -4387,32 +4375,32 @@
         </is>
       </c>
       <c r="L74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:33</t>
+          <t>2026-05-28T09:14:07</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>12311</v>
+        <v>13035</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Pindamonhangaba</t>
+          <t>Secretaria de Estado da Fazenda do Para</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Chefe de gabinete</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4420,17 +4408,21 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>Bandeirantes de Comunicação</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>sefaouvidoria@sefa.pa.gov.br; atendimento@sefa.pa.gov.br</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>(91) 3039-8549; (91) 3323-4200</t>
+        </is>
+      </c>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.pindamonhangaba.sp.gov.br/gabinete</t>
+          <t>https://www.sefa.pa.gov.br/fale-conosco</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -4439,32 +4431,32 @@
         </is>
       </c>
       <c r="L75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:36</t>
+          <t>2026-05-28T09:14:10</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>12503</v>
+        <v>13040</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Rio Claro</t>
+          <t>Secretaria de Turismo e Desenvolvimento Economico da Paraiba</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Planejamento</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4472,21 +4464,21 @@
           <t>Encontrado</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>Bruno Oliveira</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>(19) 3522-1998</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>setdegabinete@setd.pb.gov.br</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>(83) 99163-6715</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>https://rioclaro.sp.gov.br/secretaria/secretaria-de-planejamento/</t>
+          <t>https://paraiba.pb.gov.br/diretas/secretaria-de-turismo-e-desenvolvimento-economico/pagina-inicial</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -4500,53 +4492,45 @@
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:39</t>
+          <t>2026-05-28T09:14:15</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>12520</v>
+        <v>13053</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Rio das Pedras</t>
+          <t>Secretaria de Desenvolvimento Economico de Pernambuco</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Encontrado</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Marcos Buzetto</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>prefeito@riodaspedras.sp.gov.br</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>(19) 3493-9490</t>
+          <t>(81) 3182-1700; 3182-1728</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
-          <t>https://www.riodaspedras.sp.gov.br/prefeito.php?page_no=10&amp;FiltroSecretaria=8</t>
+          <t>https://www.sdec.pe.gov.br/dialogue-conosco</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -4555,32 +4539,32 @@
         </is>
       </c>
       <c r="L77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:44</t>
+          <t>2026-05-28T09:14:18</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>12564</v>
+        <v>13064</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Rio das Pedras</t>
+          <t>Secretaria de Estado do Desenvolvimento Economico do Piaui</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Vice-prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4590,19 +4574,19 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Trudpert Alan Leite Riesterer</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>9747-4700</t>
-        </is>
-      </c>
+          <t>Deusval Lacerda de Moraes</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>sde@sde.pi.gov.br</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
-          <t>https://www.riodaspedras.sp.gov.br/departamentos.php?FiltroSecretaria=25</t>
+          <t>https://www.pi.gov.br/orgao/secretaria-de-estado-do-desenvolvimento-economico-sde/</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -4616,22 +4600,22 @@
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:48</t>
+          <t>2026-05-28T09:14:24</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>12718</v>
+        <v>13107</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Sorocaba</t>
+          <t>Secretaria de Estado da Fazenda de Roraima</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4647,14 +4631,18 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>sefaz@sorocaba.sp.gov.br</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr"/>
+          <t>gabinete@sefaz.rr.gov.br; cetif@sefaz.rr.gov.br; valdeildo.menezes@sefaz.rr.gov.br</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>(95) 2121-9003; 2121-9014; 2121-9066; (95) 2121-9018; 2121-9052; 2121-9046</t>
+        </is>
+      </c>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>https://fazenda.sorocaba.sp.gov.br/</t>
+          <t>https://www.sefaz.rr.gov.br/asecretaria/aestrutura</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -4663,50 +4651,54 @@
         </is>
       </c>
       <c r="L79" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:50</t>
+          <t>2026-05-28T09:14:28</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>12783</v>
+        <v>13114</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>São Bernardo do Campo</t>
+          <t>Secretaria da Fazenda do Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Finanças/Fazenda</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Marcelo Lima</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+          <t>Encontrado</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>tesouro@sefaz.rs.gov.br; cage@sefaz.rs.gov.br</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>(51) 3214-5000; (51) 3214-5200</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
-          <t>https://www.saobernardo.sp.gov.br/web/sbc/home/-/asset_publisher/1ZeTEZMaamL4/content/em-sao-bernardo-centro-de-excelencia-do-judo-recebe-equipe-da-republica-dominicana-para-treinamento-em-conjunto/maximized?inheritRedirect=false&amp;redirect=https%3A%2F%2Fwww.saobernardo.sp.gov.br%2Fweb%2Fsbc%2Fhome%3Fp_p_id%3D101_INSTANCE_1ZeTEZMaamL4%26p_p_lifecycle%3D0%26p_p_state%3Dnormal%26p_p_mode%3Dview%26p_p_col_id%3D_118_INSTANCE_9UnxBzXMepRr__column-1%26p_p_col_count%3D1</t>
+          <t>https://fazenda.rs.gov.br/fale-conosco</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -4715,50 +4707,58 @@
         </is>
       </c>
       <c r="L80" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:53</t>
+          <t>2026-05-28T09:14:34</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>12992</v>
+        <v>13150</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Tupã</t>
+          <t>Secretaria da Industria, Comercio e Servicos do Tocantins</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Prefeito</t>
+          <t>Desenvolvimento econômico</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Encontrado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>prefeito@tupa.sp.gov.br</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
+          <t>gabinete@sics.to.gov.br; enilengenheiro@gmail.com; ezequias.monteiro@hotmail.com; wesleygabinete2012@gmail.com; luiz_filho22@hotmail.com; fabiopiau@hotmail.com; sergionbarbosajus@gmail.com; carlos.carneiro@sics.to.gov.br; joao.silva@sics.to.gov.br; vera.thoma@gmail.com; ascom@sics.to.gov.br; renatogoiababucar@gmail.com; suzanapinheiro@outlook.com; elaticosta@gmail.com; edith.tedescoreis@gmail.com; mirellanoronha@gmail.com; rh@sics.to; contabilidade@sics.to.gov.br</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>9262-7117; 9217-9666; 8451-5029; 8415-0023; 8432-2166; 8113-5027; 9997-5267</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>(11) 94847-1308; (63) 98407-9097; (63) 99936-3322; (63) 99254-8587; (63) 99914-6027; (63) 98432-8374; (63) 98403-2075</t>
+        </is>
+      </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.tupa.sp.gov.br/prefeitura/detalhe-departamento/63/prefeito/</t>
+          <t>https://www.to.gov.br/sics/lista-de-contatos/2j100aur405s</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -4767,12 +4767,12 @@
         </is>
       </c>
       <c r="L81" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr">
         <is>
-          <t>2026-05-28T04:59:57</t>
+          <t>2026-05-28T09:14:37</t>
         </is>
       </c>
     </row>

</xml_diff>